<commit_message>
Add World Cup 2026 prediction dashboard with responsive match grid.
Reorganize fixtures into expandable rounds with group cards, improve leaderboard and prediction handling, add display aliases for long team names, and load FIFA 2026 match data.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/predictions.xlsx
+++ b/data/predictions.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,336 +425,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>participant_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>username</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>match_id</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>match_label</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>predicted_score_a</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>predicted_score_b</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>predicted_outcome</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>saved_at</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ewnewf</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Spain vs England</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-06-04 12:04:21</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ewnewf</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Portugal vs Netherlands</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-06-04 12:04:32</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ewnewf</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>5</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Japan vs Canada</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-06-04 12:04:37</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>P002</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>fefer</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Spain vs England</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-06-04 12:12:26</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>P002</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>fefer</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Portugal vs Netherlands</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Draw</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-06-04 15:00:49</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>P002</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>fefer</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Japan vs Canada</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-06-04 12:12:38</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>MJ</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Alpha vs Beta</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-06-04 13:44:48</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>P001</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>MJ</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Demo Team A vs Demo Team B</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Draw</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-06-04 13:44:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
iclude demo and admin
</commit_message>
<xml_diff>
--- a/data/predictions.xlsx
+++ b/data/predictions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +470,294 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>9001</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Demo Lions vs Demo Tigers</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-06-06 18:33:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>9003</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Demo Sharks vs Demo Wolves</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-06-06 18:33:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>9002</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Demo Eagles vs Demo Bears</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-06-06 18:33:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>9004</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Demo Hawks vs Demo Foxes</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-06-06 18:33:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PS2</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>9001</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Demo Lions vs Demo Tigers</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-06-06 18:34:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PS2</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>9003</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Demo Sharks vs Demo Wolves</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-06-06 18:34:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PS2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9004</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Demo Hawks vs Demo Foxes</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-06-06 18:34:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PS2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>9002</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Demo Eagles vs Demo Bears</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-06-06 18:48:04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>